<commit_message>
data: add distal airway COPD paper
</commit_message>
<xml_diff>
--- a/db/cellxgene/our_marker_papers.xlsx
+++ b/db/cellxgene/our_marker_papers.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与统计" sheetId="1" r:id="Reeefa41b28244f89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="我方Marker文章" sheetId="2" r:id="R992368b9d35146a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与统计" sheetId="1" r:id="Rc0934bd7dc9c4aef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="我方Marker文章" sheetId="2" r:id="Rdf7e5e47e01e4edc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -296,7 +296,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -306,7 +306,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -316,7 +316,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -327,7 +327,7 @@
         <x:color rgb="FF1F4E78"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDEBF7"/>
         </x:patternFill>
       </x:fill>
@@ -338,7 +338,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -639,7 +639,7 @@
       </x:c>
       <x:c r="E4" s="31" t="n">
         <x:f>COUNTIF('我方Marker文章'!$P$2:$P$45,"已核验")</x:f>
-        <x:v>38</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F4" s="41"/>
       <x:c r="G4" s="19" t="str">
@@ -664,7 +664,7 @@
       </x:c>
       <x:c r="E5" s="32" t="n">
         <x:f>COUNTIF('我方Marker文章'!$P$2:$P$45,"缺有效PDF")+COUNTIF('我方Marker文章'!$P$2:$P$45,"求助中：缺有效PDF")</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F5" s="41"/>
       <x:c r="G5" s="21" t="str">
@@ -672,7 +672,7 @@
       </x:c>
       <x:c r="H5" s="32" t="n">
         <x:f>COUNTIF('我方Marker文章'!$S$2:$S$45,"待新版提取")</x:f>
-        <x:v>37</x:v>
+        <x:v>38</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -697,7 +697,7 @@
       </x:c>
       <x:c r="H6" s="33" t="n">
         <x:f>COUNTIF('我方Marker文章'!$S$2:$S$45,"阻塞：缺有效PDF")+COUNTIF('我方Marker文章'!$S$2:$S$45,"阻塞：需补PDF/接入")</x:f>
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1297,17 +1297,19 @@
         <x:v>10x 3' v2|10x 3' v3</x:v>
       </x:c>
       <x:c r="P7" s="51" t="str">
-        <x:v>缺有效PDF</x:v>
-      </x:c>
-      <x:c r="Q7" s="46" t="str"/>
+        <x:v>已核验</x:v>
+      </x:c>
+      <x:c r="Q7" s="46" t="str">
+        <x:v>D:/OneDrive/Desktop/组/db/cellxgene/cellxgene_filtered/downloads/PMID_36796082_A Unique Cellular Organization of Human Distal Airways and Its Disarray in Chronic Obstructive Pulmonary Disease.pdf</x:v>
+      </x:c>
       <x:c r="R7" s="45" t="str">
         <x:v>DOI_10.1164_rccm.202207-1384oc</x:v>
       </x:c>
       <x:c r="S7" s="51" t="str">
-        <x:v>阻塞：缺有效PDF</x:v>
+        <x:v>待新版提取</x:v>
       </x:c>
       <x:c r="T7" s="46" t="str">
-        <x:v>登记有论文身份，但当前有效 PDF 库缺失</x:v>
+        <x:v>官网直接下载；按用户要求未做正文复核</x:v>
       </x:c>
       <x:c r="U7" s="53" t="n">
         <x:v>41</x:v>
@@ -3707,7 +3709,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe19fc0108e6416f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b4d29de78974566"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: update reviewed marker tables
</commit_message>
<xml_diff>
--- a/db/cellxgene/our_marker_papers.xlsx
+++ b/db/cellxgene/our_marker_papers.xlsx
@@ -697,7 +697,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
@@ -819,7 +818,6 @@
         <v/>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="35" t="inlineStr">
         <is>
@@ -862,7 +860,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="40" t="inlineStr">
         <is>
@@ -1136,7 +1133,7 @@
       </c>
       <c r="T2" s="46" t="inlineStr">
         <is>
-          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查</t>
+          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查；Markdown定向复核未发现作者直接给出的正式PNS marker</t>
         </is>
       </c>
       <c r="U2" s="61" t="n">
@@ -1433,7 +1430,7 @@
       </c>
       <c r="T5" s="46" t="inlineStr">
         <is>
-          <t>旧结果不可复用：旧结果存在已确认的论文映射污染，未复用</t>
+          <t>旧结果不可复用：旧结果存在已确认的论文映射污染，未复用；Markdown定向复核未发现作者直接给出的正式PNS marker</t>
         </is>
       </c>
       <c r="U5" s="61" t="n">
@@ -1737,12 +1734,12 @@
       </c>
       <c r="S8" s="51" t="inlineStr">
         <is>
-          <t>待新版提取</t>
+          <t>新版机器提取完成，待人工复核</t>
         </is>
       </c>
       <c r="T8" s="46" t="inlineStr">
         <is>
-          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查</t>
+          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查；Markdown提及PNS细胞，但marker可能位于图表/补充材料，暂不强行录入</t>
         </is>
       </c>
       <c r="U8" s="61" t="n">
@@ -1845,7 +1842,7 @@
       </c>
       <c r="T9" s="46" t="inlineStr">
         <is>
-          <t>旧结果不可复用：旧结果存在已确认的论文映射污染，未复用</t>
+          <t>旧结果不可复用：旧结果存在已确认的论文映射污染，未复用；Markdown定向复核未发现作者直接给出的正式PNS marker</t>
         </is>
       </c>
       <c r="U9" s="61" t="n">
@@ -1943,12 +1940,12 @@
       </c>
       <c r="S10" s="51" t="inlineStr">
         <is>
-          <t>待新版提取</t>
+          <t>快速复核已录入</t>
         </is>
       </c>
       <c r="T10" s="46" t="inlineStr">
         <is>
-          <t>旧结果不可复用：未找到可复用的旧复核 CSV</t>
+          <t>旧结果不可复用：未找到可复用的旧复核 CSV；GLM预筛+Markdown定向复核录入4条；已剔除窗口误配</t>
         </is>
       </c>
       <c r="U10" s="61" t="n">
@@ -2145,12 +2142,12 @@
       </c>
       <c r="S12" s="51" t="inlineStr">
         <is>
-          <t>待新版提取</t>
+          <t>新版机器提取完成，待人工复核</t>
         </is>
       </c>
       <c r="T12" s="46" t="inlineStr">
         <is>
-          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查</t>
+          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查；Markdown提及PNS细胞，但marker可能位于图表/补充材料，暂不强行录入</t>
         </is>
       </c>
       <c r="U12" s="61" t="n">
@@ -2248,12 +2245,12 @@
       </c>
       <c r="S13" s="51" t="inlineStr">
         <is>
-          <t>待新版提取</t>
+          <t>快速复核已录入</t>
         </is>
       </c>
       <c r="T13" s="46" t="inlineStr">
         <is>
-          <t>旧结果不可复用：旧结果存在已确认的论文映射污染，未复用</t>
+          <t>旧结果不可复用：旧结果存在已确认的论文映射污染，未复用；GLM预筛+Markdown定向复核录入3条；已剔除窗口误配</t>
         </is>
       </c>
       <c r="U13" s="61" t="n">
@@ -2356,7 +2353,7 @@
       </c>
       <c r="T14" s="46" t="inlineStr">
         <is>
-          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查</t>
+          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查；Markdown定向复核未发现作者直接给出的正式PNS marker</t>
         </is>
       </c>
       <c r="U14" s="61" t="n">
@@ -2557,12 +2554,12 @@
       </c>
       <c r="S16" s="51" t="inlineStr">
         <is>
-          <t>待新版提取</t>
+          <t>新版机器提取完成，待人工复核</t>
         </is>
       </c>
       <c r="T16" s="46" t="inlineStr">
         <is>
-          <t>旧结果不可复用：未找到可复用的旧复核 CSV</t>
+          <t>旧结果不可复用：未找到可复用的旧复核 CSV；Markdown提及PNS细胞，但marker可能位于图表/补充材料，暂不强行录入</t>
         </is>
       </c>
       <c r="U16" s="61" t="n">
@@ -2665,7 +2662,7 @@
       </c>
       <c r="T17" s="46" t="inlineStr">
         <is>
-          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查</t>
+          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查；Markdown定向复核未发现作者直接给出的正式PNS marker</t>
         </is>
       </c>
       <c r="U17" s="61" t="n">
@@ -2763,12 +2760,12 @@
       </c>
       <c r="S18" s="51" t="inlineStr">
         <is>
-          <t>待新版提取</t>
+          <t>新版机器提取完成，待人工复核</t>
         </is>
       </c>
       <c r="T18" s="46" t="inlineStr">
         <is>
-          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查</t>
+          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查；Markdown提及PNS细胞，但marker可能位于图表/补充材料，暂不强行录入</t>
         </is>
       </c>
       <c r="U18" s="61" t="n">
@@ -2871,7 +2868,7 @@
       </c>
       <c r="T19" s="46" t="inlineStr">
         <is>
-          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查</t>
+          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查；Markdown定向复核未发现作者直接给出的正式PNS marker</t>
         </is>
       </c>
       <c r="U19" s="61" t="n">
@@ -3060,12 +3057,12 @@
       </c>
       <c r="S21" s="51" t="inlineStr">
         <is>
-          <t>待新版提取</t>
+          <t>新版机器提取完成，待人工复核</t>
         </is>
       </c>
       <c r="T21" s="46" t="inlineStr">
         <is>
-          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查</t>
+          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查；Markdown提及PNS细胞，但marker可能位于图表/补充材料，暂不强行录入</t>
         </is>
       </c>
       <c r="U21" s="61" t="n">
@@ -3159,12 +3156,12 @@
       </c>
       <c r="S22" s="51" t="inlineStr">
         <is>
-          <t>待新版提取</t>
+          <t>快速复核已录入</t>
         </is>
       </c>
       <c r="T22" s="46" t="inlineStr">
         <is>
-          <t>旧结果不可复用：未找到可复用的旧复核 CSV</t>
+          <t>旧结果不可复用：未找到可复用的旧复核 CSV；GLM预筛+Markdown定向复核录入2条；已剔除窗口误配</t>
         </is>
       </c>
       <c r="U22" s="61" t="n">
@@ -3267,7 +3264,7 @@
       </c>
       <c r="T23" s="46" t="inlineStr">
         <is>
-          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查</t>
+          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查；Markdown定向复核未发现作者直接给出的正式PNS marker</t>
         </is>
       </c>
       <c r="U23" s="61" t="n">
@@ -3468,12 +3465,12 @@
       </c>
       <c r="S25" s="51" t="inlineStr">
         <is>
-          <t>待新版提取</t>
+          <t>快速复核已录入</t>
         </is>
       </c>
       <c r="T25" s="46" t="inlineStr">
         <is>
-          <t>旧结果不可复用：未找到可复用的旧复核 CSV</t>
+          <t>旧结果不可复用：未找到可复用的旧复核 CSV；GLM预筛+Markdown定向复核录入2条；已剔除窗口误配</t>
         </is>
       </c>
       <c r="U25" s="61" t="n">
@@ -3877,7 +3874,7 @@
       </c>
       <c r="T29" s="46" t="inlineStr">
         <is>
-          <t>旧结果不可复用：未找到可复用的旧复核 CSV</t>
+          <t>旧结果不可复用：未找到可复用的旧复核 CSV；Markdown定向复核未发现作者直接给出的正式PNS marker</t>
         </is>
       </c>
       <c r="U29" s="61" t="n">
@@ -3980,7 +3977,7 @@
       </c>
       <c r="T30" s="46" t="inlineStr">
         <is>
-          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查</t>
+          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查；Markdown定向复核未发现作者直接给出的正式PNS marker</t>
         </is>
       </c>
       <c r="U30" s="61" t="n">
@@ -4083,7 +4080,7 @@
       </c>
       <c r="T31" s="46" t="inlineStr">
         <is>
-          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查</t>
+          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查；Markdown定向复核未发现作者直接给出的正式PNS marker</t>
         </is>
       </c>
       <c r="U31" s="61" t="n">
@@ -4289,7 +4286,7 @@
       </c>
       <c r="T33" s="46" t="inlineStr">
         <is>
-          <t>旧结果不可复用：旧结果存在已确认的论文映射污染，未复用</t>
+          <t>旧结果不可复用：旧结果存在已确认的论文映射污染，未复用；Markdown定向复核未发现作者直接给出的正式PNS marker</t>
         </is>
       </c>
       <c r="U33" s="61" t="n">
@@ -4387,12 +4384,12 @@
       </c>
       <c r="S34" s="51" t="inlineStr">
         <is>
-          <t>待新版提取</t>
+          <t>新版机器提取完成，待人工复核</t>
         </is>
       </c>
       <c r="T34" s="46" t="inlineStr">
         <is>
-          <t>旧结果不可复用：未找到可复用的旧复核 CSV</t>
+          <t>旧结果不可复用：未找到可复用的旧复核 CSV；Markdown提及PNS细胞，但marker可能位于图表/补充材料，暂不强行录入</t>
         </is>
       </c>
       <c r="U34" s="61" t="n">
@@ -4495,7 +4492,7 @@
       </c>
       <c r="T35" s="46" t="inlineStr">
         <is>
-          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查</t>
+          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查；Markdown定向复核未发现作者直接给出的正式PNS marker</t>
         </is>
       </c>
       <c r="U35" s="61" t="n">
@@ -4598,7 +4595,7 @@
       </c>
       <c r="T36" s="46" t="inlineStr">
         <is>
-          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查</t>
+          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查；Markdown定向复核未发现作者直接给出的正式PNS marker</t>
         </is>
       </c>
       <c r="U36" s="61" t="n">
@@ -4977,12 +4974,12 @@
       </c>
       <c r="S40" s="51" t="inlineStr">
         <is>
-          <t>待新版提取</t>
+          <t>新版机器提取完成，待人工复核</t>
         </is>
       </c>
       <c r="T40" s="46" t="inlineStr">
         <is>
-          <t>旧结果不可复用：旧结果存在已确认的论文映射污染，未复用</t>
+          <t>旧结果不可复用：旧结果存在已确认的论文映射污染，未复用；Markdown提及PNS细胞，但marker可能位于图表/补充材料，暂不强行录入</t>
         </is>
       </c>
       <c r="U40" s="61" t="n">
@@ -5085,7 +5082,7 @@
       </c>
       <c r="T41" s="46" t="inlineStr">
         <is>
-          <t>旧结果不可复用：未找到可复用的旧复核 CSV</t>
+          <t>旧结果不可复用：未找到可复用的旧复核 CSV；Markdown定向复核未发现作者直接给出的正式PNS marker</t>
         </is>
       </c>
       <c r="U41" s="61" t="n">
@@ -5394,7 +5391,7 @@
       </c>
       <c r="T44" s="46" t="inlineStr">
         <is>
-          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查</t>
+          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查；Markdown定向复核未发现作者直接给出的正式PNS marker</t>
         </is>
       </c>
       <c r="U44" s="61" t="n">
@@ -5497,7 +5494,7 @@
       </c>
       <c r="T45" s="46" t="inlineStr">
         <is>
-          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查</t>
+          <t>快速筛查旧结果未发现可直接录入的正式PNS marker；保留待新版提取/补查；Markdown定向复核未发现作者直接给出的正式PNS marker</t>
         </is>
       </c>
       <c r="U45" s="61" t="n">

</xml_diff>